<commit_message>
recode CoA: Equity 1xxx, Assets 3xxx; regenerate all outputs
Block-coding reshuffle to match Schedule III presentation order:
- Asset ledgers: +2000 (1xxx -> 3xxx)
- Equity ledgers: -2000 (3xxx -> 1xxx)
- Liabilities (2xxx), Income (4xxx), Expenses (5xxx-8xxx) unchanged
- Docstring and section-header comments updated to new prefixes
- All six generators re-run; 208 unique codes, all integrity checks pass

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/chart_of_accounts.xlsx
+++ b/output/chart_of_accounts.xlsx
@@ -526,7 +526,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
@@ -559,7 +559,7 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>3001</v>
+        <v>1001</v>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
@@ -592,7 +592,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>3010</v>
+        <v>1010</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>3020</v>
+        <v>1020</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
@@ -658,7 +658,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>3021</v>
+        <v>1021</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -691,7 +691,7 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>3030</v>
+        <v>1030</v>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
@@ -724,7 +724,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>3040</v>
+        <v>1040</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
@@ -757,7 +757,7 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>3050</v>
+        <v>1050</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
-        <v>1010</v>
+        <v>3010</v>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
@@ -2572,7 +2572,7 @@
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
-        <v>1015</v>
+        <v>3015</v>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
@@ -2605,7 +2605,7 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
-        <v>1020</v>
+        <v>3020</v>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
-        <v>1025</v>
+        <v>3025</v>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
@@ -2671,7 +2671,7 @@
     </row>
     <row r="68">
       <c r="A68" s="5" t="n">
-        <v>1030</v>
+        <v>3030</v>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
@@ -2704,7 +2704,7 @@
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
-        <v>1035</v>
+        <v>3035</v>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
@@ -2737,7 +2737,7 @@
     </row>
     <row r="70">
       <c r="A70" s="5" t="n">
-        <v>1040</v>
+        <v>3040</v>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
@@ -2770,7 +2770,7 @@
     </row>
     <row r="71">
       <c r="A71" s="3" t="n">
-        <v>1045</v>
+        <v>3045</v>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
@@ -2803,7 +2803,7 @@
     </row>
     <row r="72">
       <c r="A72" s="5" t="n">
-        <v>1050</v>
+        <v>3050</v>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
@@ -2836,7 +2836,7 @@
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
-        <v>1055</v>
+        <v>3055</v>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
@@ -2869,7 +2869,7 @@
     </row>
     <row r="74">
       <c r="A74" s="5" t="n">
-        <v>1060</v>
+        <v>3060</v>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
@@ -2902,7 +2902,7 @@
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
-        <v>1065</v>
+        <v>3065</v>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
     </row>
     <row r="76">
       <c r="A76" s="5" t="n">
-        <v>1070</v>
+        <v>3070</v>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
@@ -2968,7 +2968,7 @@
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
-        <v>1075</v>
+        <v>3075</v>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
@@ -3001,7 +3001,7 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="n">
-        <v>1080</v>
+        <v>3080</v>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
@@ -3034,7 +3034,7 @@
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
-        <v>1085</v>
+        <v>3085</v>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
@@ -3067,7 +3067,7 @@
     </row>
     <row r="80">
       <c r="A80" s="5" t="n">
-        <v>1100</v>
+        <v>3100</v>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
@@ -3100,7 +3100,7 @@
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
-        <v>1105</v>
+        <v>3105</v>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
-        <v>1110</v>
+        <v>3110</v>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
@@ -3166,7 +3166,7 @@
     </row>
     <row r="83">
       <c r="A83" s="3" t="n">
-        <v>1120</v>
+        <v>3120</v>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
@@ -3199,7 +3199,7 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
-        <v>1121</v>
+        <v>3121</v>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
@@ -3232,7 +3232,7 @@
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
-        <v>1125</v>
+        <v>3125</v>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
@@ -3265,7 +3265,7 @@
     </row>
     <row r="86">
       <c r="A86" s="5" t="n">
-        <v>1150</v>
+        <v>3150</v>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
@@ -3298,7 +3298,7 @@
     </row>
     <row r="87">
       <c r="A87" s="3" t="n">
-        <v>1151</v>
+        <v>3151</v>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
@@ -3331,7 +3331,7 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="n">
-        <v>1160</v>
+        <v>3160</v>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
@@ -3364,7 +3364,7 @@
     </row>
     <row r="89">
       <c r="A89" s="3" t="n">
-        <v>1170</v>
+        <v>3170</v>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
@@ -3397,7 +3397,7 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="n">
-        <v>1200</v>
+        <v>3200</v>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
@@ -3430,7 +3430,7 @@
     </row>
     <row r="91">
       <c r="A91" s="3" t="n">
-        <v>1201</v>
+        <v>3201</v>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
@@ -3463,7 +3463,7 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="n">
-        <v>1205</v>
+        <v>3205</v>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
@@ -3496,7 +3496,7 @@
     </row>
     <row r="93">
       <c r="A93" s="3" t="n">
-        <v>1210</v>
+        <v>3210</v>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
@@ -3529,7 +3529,7 @@
     </row>
     <row r="94">
       <c r="A94" s="5" t="n">
-        <v>1300</v>
+        <v>3300</v>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
-        <v>1301</v>
+        <v>3301</v>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="96">
       <c r="A96" s="5" t="n">
-        <v>1302</v>
+        <v>3302</v>
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
@@ -3628,7 +3628,7 @@
     </row>
     <row r="97">
       <c r="A97" s="3" t="n">
-        <v>1303</v>
+        <v>3303</v>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
@@ -3661,7 +3661,7 @@
     </row>
     <row r="98">
       <c r="A98" s="5" t="n">
-        <v>1304</v>
+        <v>3304</v>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
@@ -3694,7 +3694,7 @@
     </row>
     <row r="99">
       <c r="A99" s="3" t="n">
-        <v>1305</v>
+        <v>3305</v>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
@@ -3727,7 +3727,7 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="n">
-        <v>1320</v>
+        <v>3320</v>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
@@ -3760,7 +3760,7 @@
     </row>
     <row r="101">
       <c r="A101" s="3" t="n">
-        <v>1325</v>
+        <v>3325</v>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
@@ -3793,7 +3793,7 @@
     </row>
     <row r="102">
       <c r="A102" s="5" t="n">
-        <v>1330</v>
+        <v>3330</v>
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
@@ -3826,7 +3826,7 @@
     </row>
     <row r="103">
       <c r="A103" s="3" t="n">
-        <v>1335</v>
+        <v>3335</v>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
@@ -3859,7 +3859,7 @@
     </row>
     <row r="104">
       <c r="A104" s="5" t="n">
-        <v>1400</v>
+        <v>3400</v>
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
@@ -3892,7 +3892,7 @@
     </row>
     <row r="105">
       <c r="A105" s="3" t="n">
-        <v>1401</v>
+        <v>3401</v>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
@@ -3925,7 +3925,7 @@
     </row>
     <row r="106">
       <c r="A106" s="5" t="n">
-        <v>1402</v>
+        <v>3402</v>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
     </row>
     <row r="107">
       <c r="A107" s="3" t="n">
-        <v>1403</v>
+        <v>3403</v>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
@@ -3991,7 +3991,7 @@
     </row>
     <row r="108">
       <c r="A108" s="5" t="n">
-        <v>1404</v>
+        <v>3404</v>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
@@ -4024,7 +4024,7 @@
     </row>
     <row r="109">
       <c r="A109" s="3" t="n">
-        <v>1405</v>
+        <v>3405</v>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
@@ -4057,7 +4057,7 @@
     </row>
     <row r="110">
       <c r="A110" s="5" t="n">
-        <v>1406</v>
+        <v>3406</v>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
@@ -4090,7 +4090,7 @@
     </row>
     <row r="111">
       <c r="A111" s="3" t="n">
-        <v>1407</v>
+        <v>3407</v>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     </row>
     <row r="112">
       <c r="A112" s="5" t="n">
-        <v>1408</v>
+        <v>3408</v>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
@@ -4156,7 +4156,7 @@
     </row>
     <row r="113">
       <c r="A113" s="3" t="n">
-        <v>1409</v>
+        <v>3409</v>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
@@ -4189,7 +4189,7 @@
     </row>
     <row r="114">
       <c r="A114" s="5" t="n">
-        <v>1410</v>
+        <v>3410</v>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
@@ -4222,7 +4222,7 @@
     </row>
     <row r="115">
       <c r="A115" s="3" t="n">
-        <v>1411</v>
+        <v>3411</v>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
@@ -4255,7 +4255,7 @@
     </row>
     <row r="116">
       <c r="A116" s="5" t="n">
-        <v>1412</v>
+        <v>3412</v>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
@@ -4288,7 +4288,7 @@
     </row>
     <row r="117">
       <c r="A117" s="3" t="n">
-        <v>1413</v>
+        <v>3413</v>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
@@ -4321,7 +4321,7 @@
     </row>
     <row r="118">
       <c r="A118" s="5" t="n">
-        <v>1414</v>
+        <v>3414</v>
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
     </row>
     <row r="119">
       <c r="A119" s="3" t="n">
-        <v>1450</v>
+        <v>3450</v>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
@@ -4387,7 +4387,7 @@
     </row>
     <row r="120">
       <c r="A120" s="5" t="n">
-        <v>1451</v>
+        <v>3451</v>
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
@@ -4420,7 +4420,7 @@
     </row>
     <row r="121">
       <c r="A121" s="3" t="n">
-        <v>1460</v>
+        <v>3460</v>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
@@ -4453,7 +4453,7 @@
     </row>
     <row r="122">
       <c r="A122" s="5" t="n">
-        <v>1461</v>
+        <v>3461</v>
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
@@ -4486,7 +4486,7 @@
     </row>
     <row r="123">
       <c r="A123" s="3" t="n">
-        <v>1462</v>
+        <v>3462</v>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
@@ -4519,7 +4519,7 @@
     </row>
     <row r="124">
       <c r="A124" s="5" t="n">
-        <v>1463</v>
+        <v>3463</v>
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
@@ -4552,7 +4552,7 @@
     </row>
     <row r="125">
       <c r="A125" s="3" t="n">
-        <v>1500</v>
+        <v>3500</v>
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
@@ -4585,7 +4585,7 @@
     </row>
     <row r="126">
       <c r="A126" s="5" t="n">
-        <v>1501</v>
+        <v>3501</v>
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
@@ -4618,7 +4618,7 @@
     </row>
     <row r="127">
       <c r="A127" s="3" t="n">
-        <v>1550</v>
+        <v>3550</v>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
@@ -4651,7 +4651,7 @@
     </row>
     <row r="128">
       <c r="A128" s="5" t="n">
-        <v>1551</v>
+        <v>3551</v>
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
@@ -4684,7 +4684,7 @@
     </row>
     <row r="129">
       <c r="A129" s="3" t="n">
-        <v>1552</v>
+        <v>3552</v>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
@@ -4717,7 +4717,7 @@
     </row>
     <row r="130">
       <c r="A130" s="5" t="n">
-        <v>1553</v>
+        <v>3553</v>
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
@@ -4750,7 +4750,7 @@
     </row>
     <row r="131">
       <c r="A131" s="3" t="n">
-        <v>1554</v>
+        <v>3554</v>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
@@ -4783,7 +4783,7 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="n">
-        <v>1555</v>
+        <v>3555</v>
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
@@ -4816,7 +4816,7 @@
     </row>
     <row r="133">
       <c r="A133" s="3" t="n">
-        <v>1560</v>
+        <v>3560</v>
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
@@ -4849,7 +4849,7 @@
     </row>
     <row r="134">
       <c r="A134" s="5" t="n">
-        <v>1561</v>
+        <v>3561</v>
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>

</xml_diff>